<commit_message>
Version 3.5, fixed an issue with extreme variaiton in estimated biomass for combined prey types containing highly variable (size-wise) species
</commit_message>
<xml_diff>
--- a/helperfiles/Sizeclass_key.xlsx
+++ b/helperfiles/Sizeclass_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhydra-my.sharepoint.com/personal/ttinker_nhydra-eco_com/Documents/SOFA2/SOFA/helperfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{441CB33B-7DFA-428E-8B93-66C504E3CC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E594F56-E40A-47B2-AE63-3117AE00CE44}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{441CB33B-7DFA-428E-8B93-66C504E3CC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9A07380-4575-4936-A866-06ACE6FB7802}"/>
   <bookViews>
-    <workbookView xWindow="4725" yWindow="1080" windowWidth="33870" windowHeight="19305" xr2:uid="{58EDC278-7532-4510-8B21-A021042D543C}"/>
+    <workbookView xWindow="8970" yWindow="1305" windowWidth="38700" windowHeight="18810" xr2:uid="{58EDC278-7532-4510-8B21-A021042D543C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -540,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0895321-839B-42DE-A004-41E02DA7DC65}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -787,7 +787,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -803,7 +803,7 @@
       </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
@@ -817,6 +817,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="3"/>
+      <c r="G18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>